<commit_message>
Resolving problems with conferences
</commit_message>
<xml_diff>
--- a/Konekcije.xlsx
+++ b/Konekcije.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aleksandra.seva\Desktop\LineFailure\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A964634-BC8B-4F57-907C-60B98274AD77}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0644FBD9-FE78-4CCC-9818-A29F994DF421}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="146">
   <si>
     <t>KOZ</t>
   </si>
@@ -353,9 +353,6 @@
   </si>
   <si>
     <t>port-3: LL_Zastita-RR_B/SJJ4 (BTM)</t>
-  </si>
-  <si>
-    <t>port-6: RR 21 (SJJ-MST)/SJJ4 (BTM)</t>
   </si>
   <si>
     <t>BUK APP</t>
@@ -1534,6 +1531,96 @@
     <xf numFmtId="49" fontId="0" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1543,6 +1630,15 @@
     <xf numFmtId="0" fontId="0" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1552,15 +1648,6 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1577,24 +1664,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1605,78 +1674,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2829,30 +2826,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="16.5" customHeight="1">
-      <c r="A1" s="129" t="s">
+      <c r="A1" s="105" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="130"/>
-      <c r="C1" s="131"/>
-      <c r="D1" s="132" t="s">
+      <c r="B1" s="106"/>
+      <c r="C1" s="107"/>
+      <c r="D1" s="108" t="s">
+        <v>114</v>
+      </c>
+      <c r="E1" s="109"/>
+      <c r="F1" s="109"/>
+      <c r="G1" s="109"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="111" t="s">
         <v>115</v>
       </c>
-      <c r="E1" s="133"/>
-      <c r="F1" s="133"/>
-      <c r="G1" s="133"/>
-      <c r="H1" s="134"/>
-      <c r="I1" s="135" t="s">
-        <v>116</v>
-      </c>
-      <c r="J1" s="136"/>
-      <c r="K1" s="136"/>
-      <c r="L1" s="136"/>
-      <c r="M1" s="137"/>
-      <c r="N1" s="111" t="s">
+      <c r="J1" s="112"/>
+      <c r="K1" s="112"/>
+      <c r="L1" s="112"/>
+      <c r="M1" s="113"/>
+      <c r="N1" s="96" t="s">
         <v>1</v>
       </c>
-      <c r="O1" s="112"/>
-      <c r="P1" s="113"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="98"/>
     </row>
     <row r="2" spans="1:16" ht="15" customHeight="1">
       <c r="A2" s="2" t="s">
@@ -2865,7 +2862,7 @@
         <v>4</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>3</v>
@@ -2922,11 +2919,11 @@
       </c>
       <c r="L3" s="5"/>
       <c r="M3" s="6"/>
-      <c r="N3" s="111" t="s">
+      <c r="N3" s="96" t="s">
         <v>1</v>
       </c>
-      <c r="O3" s="112"/>
-      <c r="P3" s="113"/>
+      <c r="O3" s="97"/>
+      <c r="P3" s="98"/>
     </row>
     <row r="4" spans="1:16" ht="15" customHeight="1">
       <c r="A4" s="18" t="s">
@@ -2990,11 +2987,11 @@
       <c r="K5" s="23"/>
       <c r="L5" s="23"/>
       <c r="M5" s="6"/>
-      <c r="N5" s="123" t="s">
+      <c r="N5" s="99" t="s">
         <v>17</v>
       </c>
-      <c r="O5" s="124"/>
-      <c r="P5" s="125"/>
+      <c r="O5" s="100"/>
+      <c r="P5" s="101"/>
     </row>
     <row r="6" spans="1:16" ht="15" customHeight="1">
       <c r="A6" s="30" t="s">
@@ -3094,11 +3091,11 @@
       <c r="K8" s="25"/>
       <c r="L8" s="25"/>
       <c r="M8" s="26"/>
-      <c r="N8" s="138" t="s">
+      <c r="N8" s="114" t="s">
         <v>27</v>
       </c>
-      <c r="O8" s="139"/>
-      <c r="P8" s="140"/>
+      <c r="O8" s="115"/>
+      <c r="P8" s="116"/>
     </row>
     <row r="9" spans="1:16" ht="15" customHeight="1">
       <c r="A9" s="44"/>
@@ -3121,7 +3118,7 @@
         <v>29</v>
       </c>
       <c r="N9" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O9" s="11" t="s">
         <v>7</v>
@@ -3168,11 +3165,11 @@
       <c r="K11" s="46"/>
       <c r="L11" s="46"/>
       <c r="M11" s="47"/>
-      <c r="N11" s="102" t="s">
+      <c r="N11" s="120" t="s">
         <v>32</v>
       </c>
-      <c r="O11" s="103"/>
-      <c r="P11" s="104"/>
+      <c r="O11" s="121"/>
+      <c r="P11" s="122"/>
     </row>
     <row r="12" spans="1:16" ht="15" customHeight="1">
       <c r="A12" s="29"/>
@@ -3218,11 +3215,11 @@
       <c r="K13" s="46"/>
       <c r="L13" s="46"/>
       <c r="M13" s="47"/>
-      <c r="N13" s="111" t="s">
+      <c r="N13" s="96" t="s">
         <v>1</v>
       </c>
-      <c r="O13" s="112"/>
-      <c r="P13" s="113"/>
+      <c r="O13" s="97"/>
+      <c r="P13" s="98"/>
     </row>
     <row r="14" spans="1:16" ht="15" customHeight="1">
       <c r="A14" s="29"/>
@@ -3268,11 +3265,11 @@
       <c r="K15" s="46"/>
       <c r="L15" s="46"/>
       <c r="M15" s="47"/>
-      <c r="N15" s="111" t="s">
+      <c r="N15" s="96" t="s">
         <v>1</v>
       </c>
-      <c r="O15" s="112"/>
-      <c r="P15" s="113"/>
+      <c r="O15" s="97"/>
+      <c r="P15" s="98"/>
     </row>
     <row r="16" spans="1:16" ht="15" customHeight="1">
       <c r="A16" s="29"/>
@@ -3330,11 +3327,11 @@
       </c>
       <c r="L17" s="5"/>
       <c r="M17" s="6"/>
-      <c r="N17" s="123" t="s">
+      <c r="N17" s="99" t="s">
         <v>17</v>
       </c>
-      <c r="O17" s="124"/>
-      <c r="P17" s="125"/>
+      <c r="O17" s="100"/>
+      <c r="P17" s="101"/>
     </row>
     <row r="18" spans="1:16" ht="15" customHeight="1">
       <c r="A18" s="29"/>
@@ -3380,11 +3377,11 @@
       <c r="K19" s="23"/>
       <c r="L19" s="23"/>
       <c r="M19" s="6"/>
-      <c r="N19" s="102" t="s">
+      <c r="N19" s="120" t="s">
         <v>32</v>
       </c>
-      <c r="O19" s="103"/>
-      <c r="P19" s="104"/>
+      <c r="O19" s="121"/>
+      <c r="P19" s="122"/>
     </row>
     <row r="20" spans="1:16" ht="15" customHeight="1">
       <c r="A20" s="29"/>
@@ -3453,16 +3450,16 @@
       <c r="P22" s="29"/>
     </row>
     <row r="23" spans="1:16" ht="16.5" customHeight="1">
-      <c r="A23" s="138" t="s">
+      <c r="A23" s="114" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="139"/>
-      <c r="C23" s="140"/>
-      <c r="D23" s="141" t="s">
+      <c r="B23" s="115"/>
+      <c r="C23" s="116"/>
+      <c r="D23" s="117" t="s">
         <v>45</v>
       </c>
-      <c r="E23" s="142"/>
-      <c r="F23" s="143"/>
+      <c r="E23" s="118"/>
+      <c r="F23" s="119"/>
       <c r="G23" s="28"/>
       <c r="H23" s="29"/>
       <c r="I23" s="29"/>
@@ -3482,7 +3479,7 @@
         <v>10</v>
       </c>
       <c r="C24" s="55" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D24" s="7"/>
       <c r="E24" s="23"/>
@@ -3506,10 +3503,10 @@
         <v>11</v>
       </c>
       <c r="C25" s="32" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D25" s="30" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E25" s="31" t="s">
         <v>3</v>
@@ -3536,7 +3533,7 @@
         <v>10</v>
       </c>
       <c r="C26" s="56" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D26" s="13"/>
       <c r="E26" s="14"/>
@@ -3560,7 +3557,7 @@
         <v>11</v>
       </c>
       <c r="C27" s="60" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D27" s="24"/>
       <c r="E27" s="25"/>
@@ -3584,10 +3581,10 @@
         <v>46</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E28" s="11" t="s">
         <v>46</v>
@@ -3643,18 +3640,18 @@
       <c r="P30" s="29"/>
     </row>
     <row r="31" spans="1:16" ht="15" customHeight="1">
-      <c r="A31" s="126" t="s">
+      <c r="A31" s="102" t="s">
         <v>47</v>
       </c>
-      <c r="B31" s="127"/>
-      <c r="C31" s="128"/>
-      <c r="D31" s="123" t="s">
+      <c r="B31" s="103"/>
+      <c r="C31" s="104"/>
+      <c r="D31" s="99" t="s">
         <v>17</v>
       </c>
-      <c r="E31" s="124"/>
-      <c r="F31" s="124"/>
-      <c r="G31" s="124"/>
-      <c r="H31" s="125"/>
+      <c r="E31" s="100"/>
+      <c r="F31" s="100"/>
+      <c r="G31" s="100"/>
+      <c r="H31" s="101"/>
       <c r="I31" s="51"/>
       <c r="J31" s="53"/>
       <c r="K31" s="53"/>
@@ -3685,11 +3682,11 @@
       </c>
       <c r="G32" s="5"/>
       <c r="H32" s="6"/>
-      <c r="I32" s="99" t="s">
+      <c r="I32" s="132" t="s">
         <v>50</v>
       </c>
-      <c r="J32" s="100"/>
-      <c r="K32" s="101"/>
+      <c r="J32" s="133"/>
+      <c r="K32" s="134"/>
       <c r="L32" s="28"/>
       <c r="M32" s="29"/>
       <c r="N32" s="29"/>
@@ -3718,7 +3715,7 @@
         <v>52</v>
       </c>
       <c r="I33" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J33" s="11" t="s">
         <v>3</v>
@@ -3753,11 +3750,11 @@
       </c>
       <c r="G34" s="5"/>
       <c r="H34" s="6"/>
-      <c r="I34" s="105" t="s">
+      <c r="I34" s="135" t="s">
         <v>56</v>
       </c>
-      <c r="J34" s="106"/>
-      <c r="K34" s="107"/>
+      <c r="J34" s="136"/>
+      <c r="K34" s="137"/>
       <c r="L34" s="28"/>
       <c r="M34" s="29"/>
       <c r="N34" s="29"/>
@@ -3780,7 +3777,7 @@
         <v>57</v>
       </c>
       <c r="I35" s="10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J35" s="11" t="s">
         <v>3</v>
@@ -3867,16 +3864,16 @@
       <c r="P39" s="29"/>
     </row>
     <row r="40" spans="1:16" ht="16.5" customHeight="1">
-      <c r="A40" s="99" t="s">
+      <c r="A40" s="132" t="s">
         <v>50</v>
       </c>
-      <c r="B40" s="100"/>
-      <c r="C40" s="101"/>
-      <c r="D40" s="99" t="s">
+      <c r="B40" s="133"/>
+      <c r="C40" s="134"/>
+      <c r="D40" s="132" t="s">
         <v>58</v>
       </c>
-      <c r="E40" s="100"/>
-      <c r="F40" s="101"/>
+      <c r="E40" s="133"/>
+      <c r="F40" s="134"/>
       <c r="G40" s="28"/>
       <c r="H40" s="29"/>
       <c r="I40" s="29"/>
@@ -3923,7 +3920,7 @@
         <v>60</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E42" s="3" t="s">
         <v>3</v>
@@ -4001,7 +3998,7 @@
         <v>63</v>
       </c>
       <c r="D45" s="30" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E45" s="31" t="s">
         <v>3</v>
@@ -4135,25 +4132,25 @@
       <c r="P51" s="29"/>
     </row>
     <row r="52" spans="1:16" ht="15" customHeight="1">
-      <c r="A52" s="102" t="s">
+      <c r="A52" s="120" t="s">
         <v>32</v>
       </c>
-      <c r="B52" s="103"/>
-      <c r="C52" s="104"/>
-      <c r="D52" s="108" t="s">
+      <c r="B52" s="121"/>
+      <c r="C52" s="122"/>
+      <c r="D52" s="138" t="s">
         <v>65</v>
       </c>
-      <c r="E52" s="109"/>
-      <c r="F52" s="109"/>
-      <c r="G52" s="109"/>
-      <c r="H52" s="110"/>
-      <c r="I52" s="111" t="s">
+      <c r="E52" s="139"/>
+      <c r="F52" s="139"/>
+      <c r="G52" s="139"/>
+      <c r="H52" s="140"/>
+      <c r="I52" s="96" t="s">
         <v>1</v>
       </c>
-      <c r="J52" s="112"/>
-      <c r="K52" s="112"/>
-      <c r="L52" s="112"/>
-      <c r="M52" s="113"/>
+      <c r="J52" s="97"/>
+      <c r="K52" s="97"/>
+      <c r="L52" s="97"/>
+      <c r="M52" s="98"/>
       <c r="N52" s="51"/>
       <c r="O52" s="53"/>
       <c r="P52" s="53"/>
@@ -4172,11 +4169,11 @@
       <c r="K53" s="79"/>
       <c r="L53" s="79"/>
       <c r="M53" s="80"/>
-      <c r="N53" s="114" t="s">
+      <c r="N53" s="129" t="s">
         <v>66</v>
       </c>
-      <c r="O53" s="115"/>
-      <c r="P53" s="116"/>
+      <c r="O53" s="130"/>
+      <c r="P53" s="131"/>
     </row>
     <row r="54" spans="1:16" ht="15" customHeight="1">
       <c r="A54" s="2" t="s">
@@ -4208,10 +4205,10 @@
         <v>11</v>
       </c>
       <c r="M54" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="N54" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="O54" s="11" t="s">
         <v>10</v>
@@ -4236,7 +4233,7 @@
         <v>69</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J55" s="3" t="s">
         <v>10</v>
@@ -4282,11 +4279,11 @@
       <c r="M56" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="N56" s="96" t="s">
+      <c r="N56" s="126" t="s">
         <v>73</v>
       </c>
-      <c r="O56" s="97"/>
-      <c r="P56" s="98"/>
+      <c r="O56" s="127"/>
+      <c r="P56" s="128"/>
     </row>
     <row r="57" spans="1:16" ht="15" customHeight="1">
       <c r="A57" s="18" t="s">
@@ -4318,10 +4315,10 @@
         <v>30</v>
       </c>
       <c r="M57" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="N57" s="10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="O57" s="11" t="s">
         <v>10</v>
@@ -4464,11 +4461,11 @@
       <c r="K62" s="46"/>
       <c r="L62" s="88"/>
       <c r="M62" s="26"/>
-      <c r="N62" s="114" t="s">
+      <c r="N62" s="129" t="s">
         <v>66</v>
       </c>
-      <c r="O62" s="115"/>
-      <c r="P62" s="116"/>
+      <c r="O62" s="130"/>
+      <c r="P62" s="131"/>
     </row>
     <row r="63" spans="1:16" ht="15" customHeight="1">
       <c r="A63" s="29"/>
@@ -4488,10 +4485,10 @@
         <v>10</v>
       </c>
       <c r="M63" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="N63" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="O63" s="11" t="s">
         <v>10</v>
@@ -4514,11 +4511,11 @@
       <c r="K64" s="23"/>
       <c r="L64" s="23"/>
       <c r="M64" s="6"/>
-      <c r="N64" s="96" t="s">
+      <c r="N64" s="126" t="s">
         <v>73</v>
       </c>
-      <c r="O64" s="97"/>
-      <c r="P64" s="98"/>
+      <c r="O64" s="127"/>
+      <c r="P64" s="128"/>
     </row>
     <row r="65" spans="1:16" ht="15" customHeight="1">
       <c r="A65" s="29"/>
@@ -4538,10 +4535,10 @@
         <v>30</v>
       </c>
       <c r="M65" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="N65" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="O65" s="11" t="s">
         <v>10</v>
@@ -4665,18 +4662,18 @@
       <c r="P71" s="29"/>
     </row>
     <row r="72" spans="1:16" ht="16.5" customHeight="1">
-      <c r="A72" s="117" t="s">
+      <c r="A72" s="141" t="s">
         <v>85</v>
       </c>
-      <c r="B72" s="118"/>
-      <c r="C72" s="119"/>
-      <c r="D72" s="114" t="s">
+      <c r="B72" s="142"/>
+      <c r="C72" s="143"/>
+      <c r="D72" s="129" t="s">
         <v>66</v>
       </c>
-      <c r="E72" s="115"/>
-      <c r="F72" s="115"/>
-      <c r="G72" s="115"/>
-      <c r="H72" s="116"/>
+      <c r="E72" s="130"/>
+      <c r="F72" s="130"/>
+      <c r="G72" s="130"/>
+      <c r="H72" s="131"/>
       <c r="I72" s="28"/>
       <c r="J72" s="29"/>
       <c r="K72" s="29"/>
@@ -4697,7 +4694,7 @@
         <v>86</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E73" s="3" t="s">
         <v>3</v>
@@ -4904,30 +4901,30 @@
       <c r="A81" s="53"/>
       <c r="B81" s="53"/>
       <c r="C81" s="89"/>
-      <c r="D81" s="111" t="s">
+      <c r="D81" s="96" t="s">
         <v>96</v>
       </c>
-      <c r="E81" s="112"/>
-      <c r="F81" s="112"/>
-      <c r="G81" s="112"/>
-      <c r="H81" s="113"/>
-      <c r="I81" s="96" t="s">
+      <c r="E81" s="97"/>
+      <c r="F81" s="97"/>
+      <c r="G81" s="97"/>
+      <c r="H81" s="98"/>
+      <c r="I81" s="126" t="s">
         <v>73</v>
       </c>
-      <c r="J81" s="97"/>
-      <c r="K81" s="97"/>
-      <c r="L81" s="97"/>
-      <c r="M81" s="98"/>
+      <c r="J81" s="127"/>
+      <c r="K81" s="127"/>
+      <c r="L81" s="127"/>
+      <c r="M81" s="128"/>
       <c r="N81" s="28"/>
       <c r="O81" s="29"/>
       <c r="P81" s="29"/>
     </row>
     <row r="82" spans="1:16" ht="15" customHeight="1">
-      <c r="A82" s="99" t="s">
+      <c r="A82" s="132" t="s">
         <v>97</v>
       </c>
-      <c r="B82" s="100"/>
-      <c r="C82" s="101"/>
+      <c r="B82" s="133"/>
+      <c r="C82" s="134"/>
       <c r="D82" s="13"/>
       <c r="E82" s="16"/>
       <c r="F82" s="3" t="s">
@@ -4980,11 +4977,11 @@
       </c>
       <c r="L83" s="25"/>
       <c r="M83" s="26"/>
-      <c r="N83" s="105" t="s">
+      <c r="N83" s="135" t="s">
         <v>56</v>
       </c>
-      <c r="O83" s="106"/>
-      <c r="P83" s="107"/>
+      <c r="O83" s="136"/>
+      <c r="P83" s="137"/>
     </row>
     <row r="84" spans="1:16" ht="15" customHeight="1">
       <c r="A84" s="10" t="s">
@@ -4994,10 +4991,10 @@
         <v>7</v>
       </c>
       <c r="C84" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E84" s="3" t="s">
         <v>10</v>
@@ -5019,7 +5016,7 @@
         <v>102</v>
       </c>
       <c r="N84" s="90" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="O84" s="90" t="s">
         <v>3</v>
@@ -5042,11 +5039,11 @@
       <c r="K85" s="23"/>
       <c r="L85" s="23"/>
       <c r="M85" s="6"/>
-      <c r="N85" s="114" t="s">
+      <c r="N85" s="129" t="s">
         <v>66</v>
       </c>
-      <c r="O85" s="115"/>
-      <c r="P85" s="116"/>
+      <c r="O85" s="130"/>
+      <c r="P85" s="131"/>
     </row>
     <row r="86" spans="1:16" ht="15" customHeight="1">
       <c r="A86" s="29"/>
@@ -5164,11 +5161,11 @@
       </c>
       <c r="L89" s="25"/>
       <c r="M89" s="26"/>
-      <c r="N89" s="99" t="s">
+      <c r="N89" s="132" t="s">
         <v>50</v>
       </c>
-      <c r="O89" s="100"/>
-      <c r="P89" s="101"/>
+      <c r="O89" s="133"/>
+      <c r="P89" s="134"/>
     </row>
     <row r="90" spans="1:16" ht="15" customHeight="1">
       <c r="A90" s="29"/>
@@ -5180,25 +5177,13 @@
       <c r="G90" s="44"/>
       <c r="H90" s="45"/>
       <c r="I90" s="91"/>
-      <c r="J90" s="31" t="s">
-        <v>30</v>
-      </c>
-      <c r="K90" s="31" t="s">
-        <v>18</v>
-      </c>
+      <c r="J90" s="31"/>
+      <c r="K90" s="31"/>
       <c r="L90" s="92"/>
-      <c r="M90" s="32" t="s">
-        <v>111</v>
-      </c>
-      <c r="N90" s="48" t="s">
-        <v>59</v>
-      </c>
-      <c r="O90" s="49" t="s">
-        <v>3</v>
-      </c>
-      <c r="P90" s="50" t="s">
-        <v>18</v>
-      </c>
+      <c r="M90" s="32"/>
+      <c r="N90" s="48"/>
+      <c r="O90" s="49"/>
+      <c r="P90" s="50"/>
     </row>
     <row r="91" spans="1:16" ht="15" customHeight="1">
       <c r="A91" s="53"/>
@@ -5214,23 +5199,23 @@
       <c r="K91" s="23"/>
       <c r="L91" s="23"/>
       <c r="M91" s="6"/>
-      <c r="N91" s="114" t="s">
+      <c r="N91" s="129" t="s">
         <v>66</v>
       </c>
-      <c r="O91" s="115"/>
-      <c r="P91" s="116"/>
+      <c r="O91" s="130"/>
+      <c r="P91" s="131"/>
     </row>
     <row r="92" spans="1:16" ht="15" customHeight="1" thickBot="1">
-      <c r="A92" s="120" t="s">
-        <v>112</v>
-      </c>
-      <c r="B92" s="121"/>
-      <c r="C92" s="122"/>
-      <c r="D92" s="99" t="s">
+      <c r="A92" s="123" t="s">
+        <v>111</v>
+      </c>
+      <c r="B92" s="124"/>
+      <c r="C92" s="125"/>
+      <c r="D92" s="132" t="s">
         <v>97</v>
       </c>
-      <c r="E92" s="100"/>
-      <c r="F92" s="101"/>
+      <c r="E92" s="133"/>
+      <c r="F92" s="134"/>
       <c r="G92" s="28"/>
       <c r="H92" s="38"/>
       <c r="I92" s="93"/>
@@ -5242,10 +5227,10 @@
       </c>
       <c r="L92" s="94"/>
       <c r="M92" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="N92" s="10" t="s">
         <v>113</v>
-      </c>
-      <c r="N92" s="10" t="s">
-        <v>114</v>
       </c>
       <c r="O92" s="11" t="s">
         <v>28</v>
@@ -5262,10 +5247,10 @@
         <v>28</v>
       </c>
       <c r="C93" s="95" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E93" s="3" t="s">
         <v>3</v>
@@ -5292,10 +5277,10 @@
         <v>3</v>
       </c>
       <c r="C94" s="50" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D94" s="48" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E94" s="49" t="s">
         <v>3</v>
@@ -5316,6 +5301,29 @@
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="N56:P56"/>
+    <mergeCell ref="D40:F40"/>
+    <mergeCell ref="N19:P19"/>
+    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="N83:P83"/>
+    <mergeCell ref="I34:K34"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="I52:M52"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="N53:P53"/>
+    <mergeCell ref="A82:C82"/>
+    <mergeCell ref="N62:P62"/>
+    <mergeCell ref="D72:H72"/>
+    <mergeCell ref="A72:C72"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="A92:C92"/>
+    <mergeCell ref="D81:H81"/>
+    <mergeCell ref="N64:P64"/>
+    <mergeCell ref="I81:M81"/>
+    <mergeCell ref="N91:P91"/>
+    <mergeCell ref="N89:P89"/>
+    <mergeCell ref="D92:F92"/>
+    <mergeCell ref="N85:P85"/>
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="N3:P3"/>
     <mergeCell ref="N17:P17"/>
@@ -5331,29 +5339,6 @@
     <mergeCell ref="N13:P13"/>
     <mergeCell ref="N15:P15"/>
     <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A92:C92"/>
-    <mergeCell ref="D81:H81"/>
-    <mergeCell ref="N64:P64"/>
-    <mergeCell ref="I81:M81"/>
-    <mergeCell ref="N91:P91"/>
-    <mergeCell ref="N89:P89"/>
-    <mergeCell ref="D92:F92"/>
-    <mergeCell ref="N85:P85"/>
-    <mergeCell ref="N56:P56"/>
-    <mergeCell ref="D40:F40"/>
-    <mergeCell ref="N19:P19"/>
-    <mergeCell ref="A52:C52"/>
-    <mergeCell ref="N83:P83"/>
-    <mergeCell ref="I34:K34"/>
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="I52:M52"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="N53:P53"/>
-    <mergeCell ref="A82:C82"/>
-    <mergeCell ref="N62:P62"/>
-    <mergeCell ref="D72:H72"/>
-    <mergeCell ref="A72:C72"/>
-    <mergeCell ref="A40:C40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape"/>

</xml_diff>